<commit_message>
Add EAC convergence index pipeline and SADC-method index
- Load and reshape the convergence workbook (tools/load_data.py)
- Threshold-based EAC index, regional summary and sigma convergence (tools/index.py)
- SADC MCI method: per-country winsorizing, pooled min-max, PCA-weighted
  sub-indices, 0.7/0.3 country index, regional mean (tools/sadc.py)
- run_index.py writes all results to outputs/eac_convergence_index.xlsx
- METHODOLOGY.md documents methods and departures from the SADC paper
- Replace old eac_index.py / data_loader.py; stop tracking __pycache__

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Macroeconomic Convergence Criteria_Submitted.xlsx
+++ b/Macroeconomic Convergence Criteria_Submitted.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26327"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lssilydion\OneDrive - Bank of Tanzania\Desktop\DATA EAC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\EAC Covergence Index\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16ACB300-6942-4B61-946B-FC084BE6AF49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" firstSheet="1" activeTab="2"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -17,7 +18,7 @@
     <sheet name="Data_EAC_Submitted and online" sheetId="5" r:id="rId3"/>
     <sheet name="Data Sources" sheetId="6" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,12 +39,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Barindirimana, Martin De Pores</author>
   </authors>
   <commentList>
-    <comment ref="AC36" authorId="0" shapeId="0">
+    <comment ref="AC36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0100-000001000000}">
       <text>
         <r>
           <rPr>
@@ -63,12 +64,12 @@
 </file>
 
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>Barindirimana, Martin De Pores</author>
   </authors>
   <commentList>
-    <comment ref="AC36" authorId="0" shapeId="0">
+    <comment ref="AC36" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
       <text>
         <r>
           <rPr>
@@ -497,7 +498,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
@@ -651,7 +652,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -698,6 +699,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E5F"/>
         <bgColor rgb="FF1F4E5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -898,7 +905,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1054,11 +1061,59 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="4" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -1074,24 +1129,41 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1100,83 +1172,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="15" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 4 2" xfId="1"/>
+    <cellStyle name="Normal 4 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1453,25 +1461,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:J77"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="15.81640625" customWidth="1"/>
+    <col min="3" max="3" width="15.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="64" t="s">
+    <row r="2" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="71" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="65"/>
-      <c r="D2" s="65"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="65"/>
-      <c r="G2" s="65"/>
-      <c r="H2" s="66"/>
-    </row>
-    <row r="3" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="73"/>
+    </row>
+    <row r="3" spans="2:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="24"/>
       <c r="C3" s="24" t="s">
         <v>0</v>
@@ -1493,8 +1501,8 @@
       </c>
       <c r="J3" s="15"/>
     </row>
-    <row r="4" spans="2:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="57" t="s">
+    <row r="4" spans="2:10" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="69" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -1520,8 +1528,8 @@
         <v>0.99999999999999978</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="57"/>
+    <row r="5" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="69"/>
       <c r="C5" s="1" t="s">
         <v>20</v>
       </c>
@@ -1543,8 +1551,8 @@
         <v>-2.7000000000000011</v>
       </c>
     </row>
-    <row r="6" spans="2:10" ht="15.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B6" s="57"/>
+    <row r="6" spans="2:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="69"/>
       <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
@@ -1568,8 +1576,8 @@
         <v>0.75336514422928502</v>
       </c>
     </row>
-    <row r="7" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B7" s="57"/>
+    <row r="7" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B7" s="69"/>
       <c r="C7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1593,8 +1601,8 @@
         <v>-1.2999999999999989</v>
       </c>
     </row>
-    <row r="8" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B8" s="57"/>
+    <row r="8" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="69"/>
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1618,8 +1626,8 @@
         <v>5.1000000000000005</v>
       </c>
     </row>
-    <row r="9" spans="2:10" ht="15.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B9" s="57"/>
+    <row r="9" spans="2:10" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B9" s="69"/>
       <c r="C9" s="1" t="s">
         <v>30</v>
       </c>
@@ -1643,8 +1651,8 @@
         <v>0.38002174157792457</v>
       </c>
     </row>
-    <row r="10" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B10" s="57"/>
+    <row r="10" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B10" s="69"/>
       <c r="C10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1668,7 +1676,7 @@
         <v>-1.5</v>
       </c>
     </row>
-    <row r="11" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B11" s="25"/>
       <c r="C11" s="27" t="s">
         <v>31</v>
@@ -1694,8 +1702,8 @@
         <v>4.4571428571428573</v>
       </c>
     </row>
-    <row r="12" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="63" t="s">
+    <row r="12" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B12" s="70" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -1721,8 +1729,8 @@
         <v>1.5241816722822037</v>
       </c>
     </row>
-    <row r="13" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B13" s="57"/>
+    <row r="13" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B13" s="69"/>
       <c r="C13" s="3" t="s">
         <v>20</v>
       </c>
@@ -1736,8 +1744,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="57"/>
+    <row r="14" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="69"/>
       <c r="C14" s="3" t="s">
         <v>10</v>
       </c>
@@ -1761,8 +1769,8 @@
         <v>1.1442184756255411</v>
       </c>
     </row>
-    <row r="15" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B15" s="57"/>
+    <row r="15" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="69"/>
       <c r="C15" s="1" t="s">
         <v>5</v>
       </c>
@@ -1786,8 +1794,8 @@
         <v>-2.0999999999999996</v>
       </c>
     </row>
-    <row r="16" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B16" s="57"/>
+    <row r="16" spans="2:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="69"/>
       <c r="C16" s="1" t="s">
         <v>6</v>
       </c>
@@ -1811,8 +1819,8 @@
         <v>-7.8329431438127086</v>
       </c>
     </row>
-    <row r="17" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B17" s="57"/>
+    <row r="17" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B17" s="69"/>
       <c r="C17" s="1" t="s">
         <v>7</v>
       </c>
@@ -1836,8 +1844,8 @@
         <v>-1.4018106666404959</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B18" s="57"/>
+    <row r="18" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="69"/>
       <c r="C18" s="1" t="s">
         <v>8</v>
       </c>
@@ -1861,7 +1869,7 @@
         <v>-4.9000000000000004</v>
       </c>
     </row>
-    <row r="19" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B19" s="25"/>
       <c r="C19" s="27" t="s">
         <v>31</v>
@@ -1887,8 +1895,8 @@
         <v>-5.0427607305156714</v>
       </c>
     </row>
-    <row r="20" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B20" s="59" t="s">
+    <row r="20" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="75" t="s">
         <v>11</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1910,8 +1918,8 @@
         <v>15.452110221624803</v>
       </c>
     </row>
-    <row r="21" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="60"/>
+    <row r="21" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="76"/>
       <c r="C21" s="1" t="s">
         <v>20</v>
       </c>
@@ -1921,8 +1929,8 @@
       <c r="G21" s="21"/>
       <c r="H21" s="21"/>
     </row>
-    <row r="22" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B22" s="60"/>
+    <row r="22" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B22" s="76"/>
       <c r="C22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1942,8 +1950,8 @@
         <v>13.377679608522008</v>
       </c>
     </row>
-    <row r="23" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B23" s="60"/>
+    <row r="23" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="76"/>
       <c r="C23" s="1" t="s">
         <v>5</v>
       </c>
@@ -1963,8 +1971,8 @@
         <v>18.2</v>
       </c>
     </row>
-    <row r="24" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B24" s="60"/>
+    <row r="24" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B24" s="76"/>
       <c r="C24" s="1" t="s">
         <v>6</v>
       </c>
@@ -1984,8 +1992,8 @@
         <v>29.9</v>
       </c>
     </row>
-    <row r="25" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B25" s="60"/>
+    <row r="25" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="76"/>
       <c r="C25" s="1" t="s">
         <v>7</v>
       </c>
@@ -2005,8 +2013,8 @@
         <v>13.700845073742409</v>
       </c>
     </row>
-    <row r="26" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B26" s="60"/>
+    <row r="26" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B26" s="76"/>
       <c r="C26" s="1" t="s">
         <v>8</v>
       </c>
@@ -2024,7 +2032,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B27" s="26"/>
       <c r="C27" s="27" t="s">
         <v>31</v>
@@ -2050,8 +2058,8 @@
         <v>16.271772483981536</v>
       </c>
     </row>
-    <row r="28" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B28" s="61" t="s">
+    <row r="28" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="77" t="s">
         <v>12</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -2073,8 +2081,8 @@
         <v>29.443934572710639</v>
       </c>
     </row>
-    <row r="29" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B29" s="62"/>
+    <row r="29" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="78"/>
       <c r="C29" s="1" t="s">
         <v>20</v>
       </c>
@@ -2084,8 +2092,8 @@
       <c r="G29" s="21"/>
       <c r="H29" s="21"/>
     </row>
-    <row r="30" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B30" s="62"/>
+    <row r="30" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B30" s="78"/>
       <c r="C30" s="1" t="s">
         <v>10</v>
       </c>
@@ -2105,8 +2113,8 @@
         <v>12.150111253180684</v>
       </c>
     </row>
-    <row r="31" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B31" s="62"/>
+    <row r="31" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B31" s="78"/>
       <c r="C31" s="1" t="s">
         <v>5</v>
       </c>
@@ -2126,8 +2134,8 @@
         <v>13.6</v>
       </c>
     </row>
-    <row r="32" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B32" s="62"/>
+    <row r="32" spans="2:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B32" s="78"/>
       <c r="C32" s="1" t="s">
         <v>6</v>
       </c>
@@ -2147,8 +2155,8 @@
         <v>196.6</v>
       </c>
     </row>
-    <row r="33" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B33" s="62"/>
+    <row r="33" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="78"/>
       <c r="C33" s="1" t="s">
         <v>7</v>
       </c>
@@ -2168,8 +2176,8 @@
         <v>22.188863389221833</v>
       </c>
     </row>
-    <row r="34" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B34" s="62"/>
+    <row r="34" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="78"/>
       <c r="C34" s="1" t="s">
         <v>8</v>
       </c>
@@ -2189,7 +2197,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="26"/>
       <c r="C35" s="27" t="s">
         <v>31</v>
@@ -2215,8 +2223,8 @@
         <v>47.330484869185518</v>
       </c>
     </row>
-    <row r="36" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B36" s="63" t="s">
+    <row r="36" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="70" t="s">
         <v>13</v>
       </c>
       <c r="C36" s="1" t="s">
@@ -2238,8 +2246,8 @@
         <v>5.82</v>
       </c>
     </row>
-    <row r="37" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B37" s="57"/>
+    <row r="37" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="69"/>
       <c r="C37" s="1" t="s">
         <v>20</v>
       </c>
@@ -2249,8 +2257,8 @@
       <c r="G37" s="21"/>
       <c r="H37" s="21"/>
     </row>
-    <row r="38" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B38" s="57"/>
+    <row r="38" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B38" s="69"/>
       <c r="C38" s="1" t="s">
         <v>10</v>
       </c>
@@ -2270,8 +2278,8 @@
         <v>10.485979166666667</v>
       </c>
     </row>
-    <row r="39" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B39" s="57"/>
+    <row r="39" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B39" s="69"/>
       <c r="C39" s="1" t="s">
         <v>5</v>
       </c>
@@ -2291,8 +2299,8 @@
         <v>9.1</v>
       </c>
     </row>
-    <row r="40" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B40" s="57"/>
+    <row r="40" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B40" s="69"/>
       <c r="C40" s="1" t="s">
         <v>6</v>
       </c>
@@ -2312,8 +2320,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="41" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B41" s="57"/>
+    <row r="41" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B41" s="69"/>
       <c r="C41" s="1" t="s">
         <v>7</v>
       </c>
@@ -2333,8 +2341,8 @@
         <v>6.0877583333333334</v>
       </c>
     </row>
-    <row r="42" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B42" s="57"/>
+    <row r="42" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="69"/>
       <c r="C42" s="1" t="s">
         <v>8</v>
       </c>
@@ -2354,7 +2362,7 @@
         <v>13.24</v>
       </c>
     </row>
-    <row r="43" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B43" s="25"/>
       <c r="C43" s="27" t="s">
         <v>31</v>
@@ -2380,8 +2388,8 @@
         <v>8.9467475000000007</v>
       </c>
     </row>
-    <row r="44" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B44" s="63" t="s">
+    <row r="44" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B44" s="70" t="s">
         <v>14</v>
       </c>
       <c r="C44" s="1" t="s">
@@ -2403,8 +2411,8 @@
         <v>6.29</v>
       </c>
     </row>
-    <row r="45" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B45" s="57"/>
+    <row r="45" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B45" s="69"/>
       <c r="C45" s="1" t="s">
         <v>20</v>
       </c>
@@ -2414,8 +2422,8 @@
       <c r="G45" s="21"/>
       <c r="H45" s="21"/>
     </row>
-    <row r="46" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B46" s="57"/>
+    <row r="46" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B46" s="69"/>
       <c r="C46" s="1" t="s">
         <v>10</v>
       </c>
@@ -2435,8 +2443,8 @@
         <v>7.2900580163212689</v>
       </c>
     </row>
-    <row r="47" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B47" s="57"/>
+    <row r="47" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B47" s="69"/>
       <c r="C47" s="1" t="s">
         <v>5</v>
       </c>
@@ -2456,8 +2464,8 @@
         <v>8.66</v>
       </c>
     </row>
-    <row r="48" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B48" s="57"/>
+    <row r="48" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B48" s="69"/>
       <c r="C48" s="1" t="s">
         <v>6</v>
       </c>
@@ -2477,8 +2485,8 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="49" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B49" s="57"/>
+    <row r="49" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B49" s="69"/>
       <c r="C49" s="1" t="s">
         <v>7</v>
       </c>
@@ -2498,8 +2506,8 @@
         <v>7.1939220437968112</v>
       </c>
     </row>
-    <row r="50" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B50" s="57"/>
+    <row r="50" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B50" s="69"/>
       <c r="C50" s="1" t="s">
         <v>8</v>
       </c>
@@ -2519,7 +2527,7 @@
         <v>10.64</v>
       </c>
     </row>
-    <row r="51" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B51" s="25"/>
       <c r="C51" s="27" t="s">
         <v>31</v>
@@ -2545,8 +2553,8 @@
         <v>6.6889966766863465</v>
       </c>
     </row>
-    <row r="52" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B52" s="63" t="s">
+    <row r="52" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B52" s="70" t="s">
         <v>15</v>
       </c>
       <c r="C52" s="1" t="s">
@@ -2568,8 +2576,8 @@
         <v>12.9</v>
       </c>
     </row>
-    <row r="53" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B53" s="57"/>
+    <row r="53" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B53" s="69"/>
       <c r="C53" s="1" t="s">
         <v>20</v>
       </c>
@@ -2579,8 +2587,8 @@
       <c r="G53" s="17"/>
       <c r="H53" s="17"/>
     </row>
-    <row r="54" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B54" s="57"/>
+    <row r="54" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B54" s="69"/>
       <c r="C54" s="1" t="s">
         <v>10</v>
       </c>
@@ -2600,8 +2608,8 @@
         <v>12.786401494756774</v>
       </c>
     </row>
-    <row r="55" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B55" s="57"/>
+    <row r="55" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B55" s="69"/>
       <c r="C55" s="1" t="s">
         <v>5</v>
       </c>
@@ -2621,8 +2629,8 @@
         <v>16.34</v>
       </c>
     </row>
-    <row r="56" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B56" s="57"/>
+    <row r="56" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B56" s="69"/>
       <c r="C56" s="1" t="s">
         <v>6</v>
       </c>
@@ -2642,8 +2650,8 @@
         <v>15.89</v>
       </c>
     </row>
-    <row r="57" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B57" s="57"/>
+    <row r="57" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B57" s="69"/>
       <c r="C57" s="1" t="s">
         <v>7</v>
       </c>
@@ -2663,8 +2671,8 @@
         <v>16.043996446789773</v>
       </c>
     </row>
-    <row r="58" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B58" s="57"/>
+    <row r="58" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B58" s="69"/>
       <c r="C58" s="1" t="s">
         <v>8</v>
       </c>
@@ -2684,7 +2692,7 @@
         <v>18.559999999999999</v>
       </c>
     </row>
-    <row r="59" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B59" s="26"/>
       <c r="C59" s="27" t="s">
         <v>31</v>
@@ -2710,8 +2718,8 @@
         <v>15.420066323591092</v>
       </c>
     </row>
-    <row r="60" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B60" s="57" t="s">
+    <row r="60" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B60" s="69" t="s">
         <v>16</v>
       </c>
       <c r="C60" s="1" t="s">
@@ -2733,8 +2741,8 @@
         <v>26.532141598119942</v>
       </c>
     </row>
-    <row r="61" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B61" s="57"/>
+    <row r="61" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B61" s="69"/>
       <c r="C61" s="1" t="s">
         <v>20</v>
       </c>
@@ -2744,8 +2752,8 @@
       <c r="G61" s="21"/>
       <c r="H61" s="21"/>
     </row>
-    <row r="62" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B62" s="57"/>
+    <row r="62" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B62" s="69"/>
       <c r="C62" s="1" t="s">
         <v>10</v>
       </c>
@@ -2765,8 +2773,8 @@
         <v>11.821499437862109</v>
       </c>
     </row>
-    <row r="63" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B63" s="57"/>
+    <row r="63" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B63" s="69"/>
       <c r="C63" s="1" t="s">
         <v>5</v>
       </c>
@@ -2786,8 +2794,8 @@
         <v>6.54</v>
       </c>
     </row>
-    <row r="64" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B64" s="57"/>
+    <row r="64" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B64" s="69"/>
       <c r="C64" s="1" t="s">
         <v>6</v>
       </c>
@@ -2807,8 +2815,8 @@
         <v>41.47</v>
       </c>
     </row>
-    <row r="65" spans="2:8" ht="15.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B65" s="57"/>
+    <row r="65" spans="2:8" ht="15.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B65" s="69"/>
       <c r="C65" s="1" t="s">
         <v>32</v>
       </c>
@@ -2828,8 +2836,8 @@
         <v>0.52458786677453961</v>
       </c>
     </row>
-    <row r="66" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B66" s="57"/>
+    <row r="66" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B66" s="69"/>
       <c r="C66" s="1" t="s">
         <v>8</v>
       </c>
@@ -2849,7 +2857,7 @@
         <v>4.66</v>
       </c>
     </row>
-    <row r="67" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B67" s="26"/>
       <c r="C67" s="27" t="s">
         <v>31</v>
@@ -2875,13 +2883,13 @@
         <v>15.258038150459432</v>
       </c>
     </row>
-    <row r="68" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="68" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B68" s="5"/>
       <c r="C68" s="5"/>
       <c r="D68" s="5"/>
       <c r="E68" s="6"/>
     </row>
-    <row r="69" spans="2:8" ht="15" x14ac:dyDescent="0.35">
+    <row r="69" spans="2:8" ht="15" x14ac:dyDescent="0.3">
       <c r="B69" s="7" t="s">
         <v>18</v>
       </c>
@@ -2889,15 +2897,15 @@
       <c r="D69" s="5"/>
       <c r="E69" s="6"/>
     </row>
-    <row r="70" spans="2:8" ht="15" x14ac:dyDescent="0.35">
-      <c r="B70" s="58" t="s">
+    <row r="70" spans="2:8" ht="15" x14ac:dyDescent="0.3">
+      <c r="B70" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="C70" s="58"/>
+      <c r="C70" s="74"/>
       <c r="D70" s="5"/>
       <c r="E70" s="6"/>
     </row>
-    <row r="71" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="71" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B71" s="10" t="s">
         <v>23</v>
       </c>
@@ -2905,37 +2913,37 @@
       <c r="D71" s="5"/>
       <c r="E71" s="5"/>
     </row>
-    <row r="72" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="72" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B72" s="5"/>
       <c r="C72" s="5"/>
       <c r="D72" s="5"/>
       <c r="E72" s="5"/>
     </row>
-    <row r="73" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="73" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B73" s="5"/>
       <c r="C73" s="5"/>
       <c r="D73" s="5"/>
       <c r="E73" s="5"/>
     </row>
-    <row r="74" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="74" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B74" s="5"/>
       <c r="C74" s="5"/>
       <c r="D74" s="5"/>
       <c r="E74" s="5"/>
     </row>
-    <row r="75" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="75" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B75" s="5"/>
       <c r="C75" s="5"/>
       <c r="D75" s="5"/>
       <c r="E75" s="5"/>
     </row>
-    <row r="76" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="76" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B76" s="5"/>
       <c r="C76" s="5"/>
       <c r="D76" s="5"/>
       <c r="E76" s="5"/>
     </row>
-    <row r="77" spans="2:8" x14ac:dyDescent="0.35">
+    <row r="77" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B77" s="5"/>
       <c r="C77" s="5"/>
       <c r="D77" s="5"/>
@@ -2943,16 +2951,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B60:B66"/>
+    <mergeCell ref="B70:C70"/>
+    <mergeCell ref="B20:B26"/>
+    <mergeCell ref="B28:B34"/>
+    <mergeCell ref="B36:B42"/>
     <mergeCell ref="B4:B10"/>
     <mergeCell ref="B12:B18"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B44:B50"/>
     <mergeCell ref="B52:B58"/>
-    <mergeCell ref="B60:B66"/>
-    <mergeCell ref="B70:C70"/>
-    <mergeCell ref="B20:B26"/>
-    <mergeCell ref="B28:B34"/>
-    <mergeCell ref="B36:B42"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2961,46 +2969,46 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:AC45"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.1796875" style="34"/>
-    <col min="2" max="2" width="31.81640625" style="34" customWidth="1"/>
-    <col min="3" max="3" width="15.1796875" style="34" customWidth="1"/>
-    <col min="4" max="29" width="12.1796875" style="34" customWidth="1"/>
-    <col min="30" max="16384" width="9.1796875" style="34"/>
+    <col min="1" max="1" width="9.21875" style="34"/>
+    <col min="2" max="2" width="31.77734375" style="34" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" style="34" customWidth="1"/>
+    <col min="4" max="29" width="12.21875" style="34" customWidth="1"/>
+    <col min="30" max="16384" width="9.21875" style="34"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:29" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B1" s="69" t="s">
+    <row r="1" spans="2:29" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B1" s="92" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="70"/>
-      <c r="S1" s="70"/>
-      <c r="T1" s="70"/>
-      <c r="U1" s="70"/>
-      <c r="V1" s="70"/>
-      <c r="W1" s="70"/>
-      <c r="X1" s="70"/>
-      <c r="Y1" s="70"/>
-    </row>
-    <row r="2" spans="2:29" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
+      <c r="H1" s="93"/>
+      <c r="I1" s="93"/>
+      <c r="J1" s="93"/>
+      <c r="K1" s="93"/>
+      <c r="L1" s="93"/>
+      <c r="M1" s="93"/>
+      <c r="N1" s="93"/>
+      <c r="O1" s="93"/>
+      <c r="P1" s="93"/>
+      <c r="Q1" s="93"/>
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="93"/>
+      <c r="U1" s="93"/>
+      <c r="V1" s="93"/>
+      <c r="W1" s="93"/>
+      <c r="X1" s="93"/>
+      <c r="Y1" s="93"/>
+    </row>
+    <row r="2" spans="2:29" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B2" s="33"/>
       <c r="C2"/>
       <c r="D2" s="54" t="s">
@@ -3030,7 +3038,7 @@
       <c r="X2"/>
       <c r="Y2"/>
     </row>
-    <row r="3" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
       <c r="D3" s="35"/>
@@ -3060,122 +3068,122 @@
       <c r="AB3" s="35"/>
       <c r="AC3" s="35"/>
     </row>
-    <row r="4" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="71"/>
-      <c r="C4" s="76" t="s">
+    <row r="4" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="94"/>
+      <c r="C4" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="67" t="s">
+      <c r="D4" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="67" t="s">
+      <c r="E4" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="67" t="s">
+      <c r="F4" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="67" t="s">
+      <c r="G4" s="79" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="67" t="s">
+      <c r="H4" s="79" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="67" t="s">
+      <c r="I4" s="79" t="s">
         <v>42</v>
       </c>
-      <c r="J4" s="67" t="s">
+      <c r="J4" s="79" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="67" t="s">
+      <c r="K4" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="67" t="s">
+      <c r="L4" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="M4" s="67" t="s">
+      <c r="M4" s="79" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="67" t="s">
+      <c r="N4" s="79" t="s">
         <v>47</v>
       </c>
-      <c r="O4" s="67" t="s">
+      <c r="O4" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="P4" s="67" t="s">
+      <c r="P4" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="Q4" s="67" t="s">
+      <c r="Q4" s="79" t="s">
         <v>50</v>
       </c>
-      <c r="R4" s="67" t="s">
+      <c r="R4" s="79" t="s">
         <v>51</v>
       </c>
-      <c r="S4" s="67" t="s">
+      <c r="S4" s="79" t="s">
         <v>52</v>
       </c>
-      <c r="T4" s="67" t="s">
+      <c r="T4" s="79" t="s">
         <v>53</v>
       </c>
-      <c r="U4" s="67" t="s">
+      <c r="U4" s="79" t="s">
         <v>54</v>
       </c>
-      <c r="V4" s="67" t="s">
+      <c r="V4" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="W4" s="67" t="s">
+      <c r="W4" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="X4" s="67" t="s">
+      <c r="X4" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="Y4" s="67" t="s">
+      <c r="Y4" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="Z4" s="67" t="s">
+      <c r="Z4" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="AA4" s="67" t="s">
+      <c r="AA4" s="79" t="s">
         <v>33</v>
       </c>
-      <c r="AB4" s="67" t="s">
+      <c r="AB4" s="79" t="s">
         <v>34</v>
       </c>
-      <c r="AC4" s="67" t="s">
+      <c r="AC4" s="79" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="72"/>
-      <c r="C5" s="76"/>
-      <c r="D5" s="68"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="68"/>
-      <c r="G5" s="68"/>
-      <c r="H5" s="68"/>
-      <c r="I5" s="68"/>
-      <c r="J5" s="68"/>
-      <c r="K5" s="68"/>
-      <c r="L5" s="68"/>
-      <c r="M5" s="68"/>
-      <c r="N5" s="68"/>
-      <c r="O5" s="68"/>
-      <c r="P5" s="68"/>
-      <c r="Q5" s="68"/>
-      <c r="R5" s="68"/>
-      <c r="S5" s="68"/>
-      <c r="T5" s="68"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="68"/>
-      <c r="W5" s="68"/>
-      <c r="X5" s="68"/>
-      <c r="Y5" s="68"/>
-      <c r="Z5" s="68"/>
-      <c r="AA5" s="68"/>
-      <c r="AB5" s="68"/>
-      <c r="AC5" s="68"/>
-    </row>
-    <row r="6" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="76" t="s">
+    <row r="5" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="95"/>
+      <c r="C5" s="81"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="80"/>
+      <c r="F5" s="80"/>
+      <c r="G5" s="80"/>
+      <c r="H5" s="80"/>
+      <c r="I5" s="80"/>
+      <c r="J5" s="80"/>
+      <c r="K5" s="80"/>
+      <c r="L5" s="80"/>
+      <c r="M5" s="80"/>
+      <c r="N5" s="80"/>
+      <c r="O5" s="80"/>
+      <c r="P5" s="80"/>
+      <c r="Q5" s="80"/>
+      <c r="R5" s="80"/>
+      <c r="S5" s="80"/>
+      <c r="T5" s="80"/>
+      <c r="U5" s="80"/>
+      <c r="V5" s="80"/>
+      <c r="W5" s="80"/>
+      <c r="X5" s="80"/>
+      <c r="Y5" s="80"/>
+      <c r="Z5" s="80"/>
+      <c r="AA5" s="80"/>
+      <c r="AB5" s="80"/>
+      <c r="AC5" s="80"/>
+    </row>
+    <row r="6" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="81" t="s">
         <v>58</v>
       </c>
       <c r="C6" s="38" t="s">
@@ -3260,8 +3268,8 @@
         <v>34.008132371032296</v>
       </c>
     </row>
-    <row r="7" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="76"/>
+    <row r="7" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="81"/>
       <c r="C7" s="38" t="s">
         <v>35</v>
       </c>
@@ -3292,8 +3300,8 @@
       <c r="AB7" s="43"/>
       <c r="AC7" s="43"/>
     </row>
-    <row r="8" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="76"/>
+    <row r="8" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="81"/>
       <c r="C8" s="38" t="s">
         <v>10</v>
       </c>
@@ -3368,8 +3376,8 @@
         <v>6.41</v>
       </c>
     </row>
-    <row r="9" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="76"/>
+    <row r="9" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="81"/>
       <c r="C9" s="39" t="s">
         <v>5</v>
       </c>
@@ -3442,8 +3450,8 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="10" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="76"/>
+    <row r="10" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="81"/>
       <c r="C10" s="39" t="s">
         <v>36</v>
       </c>
@@ -3474,8 +3482,8 @@
       <c r="AB10" s="43"/>
       <c r="AC10" s="43"/>
     </row>
-    <row r="11" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="76"/>
+    <row r="11" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="81"/>
       <c r="C11" s="39" t="s">
         <v>6</v>
       </c>
@@ -3530,8 +3538,8 @@
       <c r="AB11" s="43"/>
       <c r="AC11" s="43"/>
     </row>
-    <row r="12" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="76"/>
+    <row r="12" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="81"/>
       <c r="C12" s="39" t="s">
         <v>7</v>
       </c>
@@ -3614,8 +3622,8 @@
         <v>4.0408222020069662</v>
       </c>
     </row>
-    <row r="13" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="76"/>
+    <row r="13" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="81"/>
       <c r="C13" s="39" t="s">
         <v>8</v>
       </c>
@@ -3646,8 +3654,8 @@
       <c r="AB13" s="43"/>
       <c r="AC13" s="43"/>
     </row>
-    <row r="14" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="77"/>
+    <row r="14" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="82"/>
       <c r="C14" s="39"/>
       <c r="D14" s="44"/>
       <c r="E14" s="44"/>
@@ -3676,8 +3684,8 @@
       <c r="AB14" s="44"/>
       <c r="AC14" s="44"/>
     </row>
-    <row r="15" spans="2:29" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="81" t="s">
+    <row r="15" spans="2:29" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="86" t="s">
         <v>60</v>
       </c>
       <c r="C15" s="40" t="s">
@@ -3738,8 +3746,8 @@
         <v>2.0438541684263956</v>
       </c>
     </row>
-    <row r="16" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="82"/>
+    <row r="16" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="87"/>
       <c r="C16" s="40" t="s">
         <v>35</v>
       </c>
@@ -3770,8 +3778,8 @@
       <c r="AB16" s="46"/>
       <c r="AC16" s="46"/>
     </row>
-    <row r="17" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="82"/>
+    <row r="17" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="87"/>
       <c r="C17" s="40" t="s">
         <v>10</v>
       </c>
@@ -3826,8 +3834,8 @@
         <v>5.7681311123322816</v>
       </c>
     </row>
-    <row r="18" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="82"/>
+    <row r="18" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="87"/>
       <c r="C18" s="40" t="s">
         <v>5</v>
       </c>
@@ -3890,8 +3898,8 @@
         <v>4.1223540867584374</v>
       </c>
     </row>
-    <row r="19" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="82"/>
+    <row r="19" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="87"/>
       <c r="C19" s="40" t="s">
         <v>36</v>
       </c>
@@ -3922,8 +3930,8 @@
       <c r="AB19" s="43"/>
       <c r="AC19" s="43"/>
     </row>
-    <row r="20" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="82"/>
+    <row r="20" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="87"/>
       <c r="C20" s="40" t="s">
         <v>6</v>
       </c>
@@ -3984,8 +3992,8 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="21" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B21" s="82"/>
+    <row r="21" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="87"/>
       <c r="C21" s="40" t="s">
         <v>7</v>
       </c>
@@ -4064,8 +4072,8 @@
         <v>4.3655198743777506</v>
       </c>
     </row>
-    <row r="22" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="82"/>
+    <row r="22" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="87"/>
       <c r="C22" s="40" t="s">
         <v>8</v>
       </c>
@@ -4104,8 +4112,8 @@
         <v>3.6771878487771641</v>
       </c>
     </row>
-    <row r="23" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="83"/>
+    <row r="23" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="88"/>
       <c r="C23" s="40"/>
       <c r="D23" s="47"/>
       <c r="E23" s="47"/>
@@ -4134,8 +4142,8 @@
       <c r="AB23" s="47"/>
       <c r="AC23" s="47"/>
     </row>
-    <row r="24" spans="2:29" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="78" t="s">
+    <row r="24" spans="2:29" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="83" t="s">
         <v>59</v>
       </c>
       <c r="C24" s="39" t="s">
@@ -4198,8 +4206,8 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="25" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="79"/>
+    <row r="25" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="84"/>
       <c r="C25" s="39" t="s">
         <v>35</v>
       </c>
@@ -4230,8 +4238,8 @@
       <c r="AB25" s="51"/>
       <c r="AC25" s="51"/>
     </row>
-    <row r="26" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="79"/>
+    <row r="26" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="84"/>
       <c r="C26" s="39" t="s">
         <v>10</v>
       </c>
@@ -4314,8 +4322,8 @@
         <v>-7.2560365679833261</v>
       </c>
     </row>
-    <row r="27" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="79"/>
+    <row r="27" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="84"/>
       <c r="C27" s="39" t="s">
         <v>5</v>
       </c>
@@ -4386,8 +4394,8 @@
         <v>-5.7</v>
       </c>
     </row>
-    <row r="28" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="79"/>
+    <row r="28" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="84"/>
       <c r="C28" s="39" t="s">
         <v>36</v>
       </c>
@@ -4418,8 +4426,8 @@
       <c r="AB28" s="51"/>
       <c r="AC28" s="51"/>
     </row>
-    <row r="29" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="79"/>
+    <row r="29" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="84"/>
       <c r="C29" s="39" t="s">
         <v>6</v>
       </c>
@@ -4478,8 +4486,8 @@
         <v>2.5569999999999999</v>
       </c>
     </row>
-    <row r="30" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="79"/>
+    <row r="30" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="84"/>
       <c r="C30" s="39" t="s">
         <v>7</v>
       </c>
@@ -4562,8 +4570,8 @@
         <v>-2.5324702348127164</v>
       </c>
     </row>
-    <row r="31" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="79"/>
+    <row r="31" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="84"/>
       <c r="C31" s="39" t="s">
         <v>8</v>
       </c>
@@ -4594,8 +4602,8 @@
       <c r="AB31" s="42"/>
       <c r="AC31" s="42"/>
     </row>
-    <row r="32" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="80"/>
+    <row r="32" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="85"/>
       <c r="C32" s="39"/>
       <c r="D32" s="44"/>
       <c r="E32" s="44"/>
@@ -4624,8 +4632,8 @@
       <c r="AB32" s="44"/>
       <c r="AC32" s="44"/>
     </row>
-    <row r="33" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="73" t="s">
+    <row r="33" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="89" t="s">
         <v>61</v>
       </c>
       <c r="C33" s="40" t="s">
@@ -4690,8 +4698,8 @@
         <v>42.505624189722383</v>
       </c>
     </row>
-    <row r="34" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="74"/>
+    <row r="34" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="90"/>
       <c r="C34" s="40" t="s">
         <v>35</v>
       </c>
@@ -4722,8 +4730,8 @@
       <c r="AB34" s="46"/>
       <c r="AC34" s="46"/>
     </row>
-    <row r="35" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="74"/>
+    <row r="35" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="90"/>
       <c r="C35" s="40" t="s">
         <v>10</v>
       </c>
@@ -4806,8 +4814,8 @@
         <v>65.599999999999994</v>
       </c>
     </row>
-    <row r="36" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="74"/>
+    <row r="36" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="90"/>
       <c r="C36" s="40" t="s">
         <v>5</v>
       </c>
@@ -4862,8 +4870,8 @@
         <v>53.7</v>
       </c>
     </row>
-    <row r="37" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="74"/>
+    <row r="37" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="90"/>
       <c r="C37" s="40" t="s">
         <v>36</v>
       </c>
@@ -4894,8 +4902,8 @@
       <c r="AB37" s="43"/>
       <c r="AC37" s="43"/>
     </row>
-    <row r="38" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="74"/>
+    <row r="38" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="90"/>
       <c r="C38" s="40" t="s">
         <v>6</v>
       </c>
@@ -4954,8 +4962,8 @@
         <v>35.183846266442188</v>
       </c>
     </row>
-    <row r="39" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="74"/>
+    <row r="39" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="90"/>
       <c r="C39" s="40" t="s">
         <v>7</v>
       </c>
@@ -4986,8 +4994,8 @@
       <c r="AB39" s="43"/>
       <c r="AC39" s="43"/>
     </row>
-    <row r="40" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="74"/>
+    <row r="40" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="90"/>
       <c r="C40" s="40" t="s">
         <v>8</v>
       </c>
@@ -5018,8 +5026,8 @@
       <c r="AB40" s="42"/>
       <c r="AC40" s="42"/>
     </row>
-    <row r="41" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B41" s="75"/>
+    <row r="41" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B41" s="91"/>
       <c r="C41" s="41"/>
       <c r="D41" s="53"/>
       <c r="E41" s="53"/>
@@ -5048,7 +5056,7 @@
       <c r="AB41" s="53"/>
       <c r="AC41" s="53"/>
     </row>
-    <row r="42" spans="2:29" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:29" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="36"/>
       <c r="C42" s="37"/>
       <c r="D42" s="37"/>
@@ -5077,7 +5085,7 @@
       <c r="AB42" s="37"/>
       <c r="AC42" s="37"/>
     </row>
-    <row r="43" spans="2:29" ht="16" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:29" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B43" s="36"/>
       <c r="C43" s="37"/>
       <c r="D43" s="37"/>
@@ -5106,14 +5114,33 @@
       <c r="AB43" s="37"/>
       <c r="AC43" s="37"/>
     </row>
-    <row r="44" spans="2:29" ht="16" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:29" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B44" s="36"/>
     </row>
-    <row r="45" spans="2:29" ht="16" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:29" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B45" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="AC4:AC5"/>
+    <mergeCell ref="Y4:Y5"/>
+    <mergeCell ref="B1:Y1"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="X4:X5"/>
+    <mergeCell ref="W4:W5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="Z4:Z5"/>
+    <mergeCell ref="AA4:AA5"/>
+    <mergeCell ref="AB4:AB5"/>
+    <mergeCell ref="P4:P5"/>
+    <mergeCell ref="Q4:Q5"/>
+    <mergeCell ref="R4:R5"/>
+    <mergeCell ref="B33:B41"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="T4:T5"/>
+    <mergeCell ref="V4:V5"/>
+    <mergeCell ref="I4:I5"/>
     <mergeCell ref="U4:U5"/>
     <mergeCell ref="J4:J5"/>
     <mergeCell ref="B6:B14"/>
@@ -5128,25 +5155,6 @@
     <mergeCell ref="H4:H5"/>
     <mergeCell ref="S4:S5"/>
     <mergeCell ref="K4:K5"/>
-    <mergeCell ref="B33:B41"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="T4:T5"/>
-    <mergeCell ref="V4:V5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="AC4:AC5"/>
-    <mergeCell ref="Y4:Y5"/>
-    <mergeCell ref="B1:Y1"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="X4:X5"/>
-    <mergeCell ref="W4:W5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="Z4:Z5"/>
-    <mergeCell ref="AA4:AA5"/>
-    <mergeCell ref="AB4:AB5"/>
-    <mergeCell ref="P4:P5"/>
-    <mergeCell ref="Q4:Q5"/>
-    <mergeCell ref="R4:R5"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5156,48 +5164,48 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B1:AE45"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.21875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.1796875" style="34"/>
-    <col min="2" max="2" width="31.81640625" style="34" customWidth="1"/>
-    <col min="3" max="3" width="15.1796875" style="34" customWidth="1"/>
-    <col min="4" max="29" width="12.1796875" style="34" customWidth="1"/>
-    <col min="30" max="16384" width="9.1796875" style="34"/>
+    <col min="1" max="1" width="9.21875" style="34"/>
+    <col min="2" max="2" width="31.77734375" style="34" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" style="34" customWidth="1"/>
+    <col min="4" max="29" width="12.21875" style="34" customWidth="1"/>
+    <col min="30" max="16384" width="9.21875" style="34"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:31" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B1" s="69" t="s">
+    <row r="1" spans="2:31" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B1" s="92" t="s">
         <v>57</v>
       </c>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-      <c r="E1" s="70"/>
-      <c r="F1" s="70"/>
-      <c r="G1" s="70"/>
-      <c r="H1" s="70"/>
-      <c r="I1" s="70"/>
-      <c r="J1" s="70"/>
-      <c r="K1" s="70"/>
-      <c r="L1" s="70"/>
-      <c r="M1" s="70"/>
-      <c r="N1" s="70"/>
-      <c r="O1" s="70"/>
-      <c r="P1" s="70"/>
-      <c r="Q1" s="70"/>
-      <c r="R1" s="70"/>
-      <c r="S1" s="70"/>
-      <c r="T1" s="70"/>
-      <c r="U1" s="70"/>
-      <c r="V1" s="70"/>
-      <c r="W1" s="70"/>
-      <c r="X1" s="70"/>
-      <c r="Y1" s="70"/>
-    </row>
-    <row r="2" spans="2:31" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="B2" s="55"/>
-      <c r="C2" s="56"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
+      <c r="H1" s="93"/>
+      <c r="I1" s="93"/>
+      <c r="J1" s="93"/>
+      <c r="K1" s="93"/>
+      <c r="L1" s="93"/>
+      <c r="M1" s="93"/>
+      <c r="N1" s="93"/>
+      <c r="O1" s="93"/>
+      <c r="P1" s="93"/>
+      <c r="Q1" s="93"/>
+      <c r="R1" s="93"/>
+      <c r="S1" s="93"/>
+      <c r="T1" s="93"/>
+      <c r="U1" s="93"/>
+      <c r="V1" s="93"/>
+      <c r="W1" s="93"/>
+      <c r="X1" s="93"/>
+      <c r="Y1" s="93"/>
+    </row>
+    <row r="2" spans="2:31" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B2" s="33"/>
+      <c r="C2"/>
       <c r="D2" s="54" t="s">
         <v>56</v>
       </c>
@@ -5212,20 +5220,20 @@
       <c r="M2" s="54"/>
       <c r="N2" s="54"/>
       <c r="O2" s="54"/>
-      <c r="P2" s="56">
+      <c r="P2">
         <v>100</v>
       </c>
-      <c r="Q2" s="56"/>
-      <c r="R2" s="56"/>
-      <c r="S2" s="56"/>
-      <c r="T2" s="56"/>
-      <c r="U2" s="56"/>
-      <c r="V2" s="56"/>
-      <c r="W2" s="56"/>
-      <c r="X2" s="56"/>
-      <c r="Y2" s="56"/>
-    </row>
-    <row r="3" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="Q2"/>
+      <c r="R2"/>
+      <c r="S2"/>
+      <c r="T2"/>
+      <c r="U2"/>
+      <c r="V2"/>
+      <c r="W2"/>
+      <c r="X2"/>
+      <c r="Y2"/>
+    </row>
+    <row r="3" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
       <c r="D3" s="35"/>
@@ -5255,122 +5263,122 @@
       <c r="AB3" s="35"/>
       <c r="AC3" s="35"/>
     </row>
-    <row r="4" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="71"/>
-      <c r="C4" s="76" t="s">
+    <row r="4" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="94"/>
+      <c r="C4" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="67" t="s">
+      <c r="D4" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="67" t="s">
+      <c r="E4" s="79" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="67" t="s">
+      <c r="F4" s="79" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="67" t="s">
+      <c r="G4" s="79" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="67" t="s">
+      <c r="H4" s="79" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="67" t="s">
+      <c r="I4" s="79" t="s">
         <v>42</v>
       </c>
-      <c r="J4" s="67" t="s">
+      <c r="J4" s="79" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="67" t="s">
+      <c r="K4" s="79" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="67" t="s">
+      <c r="L4" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="M4" s="67" t="s">
+      <c r="M4" s="79" t="s">
         <v>46</v>
       </c>
-      <c r="N4" s="67" t="s">
+      <c r="N4" s="79" t="s">
         <v>47</v>
       </c>
-      <c r="O4" s="67" t="s">
+      <c r="O4" s="79" t="s">
         <v>48</v>
       </c>
-      <c r="P4" s="67" t="s">
+      <c r="P4" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="Q4" s="67" t="s">
+      <c r="Q4" s="79" t="s">
         <v>50</v>
       </c>
-      <c r="R4" s="67" t="s">
+      <c r="R4" s="79" t="s">
         <v>51</v>
       </c>
-      <c r="S4" s="67" t="s">
+      <c r="S4" s="79" t="s">
         <v>52</v>
       </c>
-      <c r="T4" s="67" t="s">
+      <c r="T4" s="79" t="s">
         <v>53</v>
       </c>
-      <c r="U4" s="67" t="s">
+      <c r="U4" s="79" t="s">
         <v>54</v>
       </c>
-      <c r="V4" s="67" t="s">
+      <c r="V4" s="79" t="s">
         <v>1</v>
       </c>
-      <c r="W4" s="67" t="s">
+      <c r="W4" s="79" t="s">
         <v>2</v>
       </c>
-      <c r="X4" s="67" t="s">
+      <c r="X4" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="Y4" s="67" t="s">
+      <c r="Y4" s="79" t="s">
         <v>22</v>
       </c>
-      <c r="Z4" s="67" t="s">
+      <c r="Z4" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="AA4" s="67" t="s">
+      <c r="AA4" s="79" t="s">
         <v>33</v>
       </c>
-      <c r="AB4" s="67" t="s">
+      <c r="AB4" s="79" t="s">
         <v>34</v>
       </c>
-      <c r="AC4" s="67" t="s">
+      <c r="AC4" s="79" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="2:31" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="72"/>
-      <c r="C5" s="76"/>
-      <c r="D5" s="68"/>
-      <c r="E5" s="68"/>
-      <c r="F5" s="68"/>
-      <c r="G5" s="68"/>
-      <c r="H5" s="68"/>
-      <c r="I5" s="68"/>
-      <c r="J5" s="68"/>
-      <c r="K5" s="68"/>
-      <c r="L5" s="68"/>
-      <c r="M5" s="68"/>
-      <c r="N5" s="68"/>
-      <c r="O5" s="68"/>
-      <c r="P5" s="68"/>
-      <c r="Q5" s="68"/>
-      <c r="R5" s="68"/>
-      <c r="S5" s="68"/>
-      <c r="T5" s="68"/>
-      <c r="U5" s="68"/>
-      <c r="V5" s="68"/>
-      <c r="W5" s="68"/>
-      <c r="X5" s="68"/>
-      <c r="Y5" s="68"/>
-      <c r="Z5" s="68"/>
-      <c r="AA5" s="68"/>
-      <c r="AB5" s="68"/>
-      <c r="AC5" s="68"/>
-    </row>
-    <row r="6" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="76" t="s">
+    <row r="5" spans="2:31" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="95"/>
+      <c r="C5" s="81"/>
+      <c r="D5" s="80"/>
+      <c r="E5" s="80"/>
+      <c r="F5" s="80"/>
+      <c r="G5" s="80"/>
+      <c r="H5" s="80"/>
+      <c r="I5" s="80"/>
+      <c r="J5" s="80"/>
+      <c r="K5" s="80"/>
+      <c r="L5" s="80"/>
+      <c r="M5" s="80"/>
+      <c r="N5" s="80"/>
+      <c r="O5" s="80"/>
+      <c r="P5" s="80"/>
+      <c r="Q5" s="80"/>
+      <c r="R5" s="80"/>
+      <c r="S5" s="80"/>
+      <c r="T5" s="80"/>
+      <c r="U5" s="80"/>
+      <c r="V5" s="80"/>
+      <c r="W5" s="80"/>
+      <c r="X5" s="80"/>
+      <c r="Y5" s="80"/>
+      <c r="Z5" s="80"/>
+      <c r="AA5" s="80"/>
+      <c r="AB5" s="80"/>
+      <c r="AC5" s="80"/>
+    </row>
+    <row r="6" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="81" t="s">
         <v>58</v>
       </c>
       <c r="C6" s="38" t="s">
@@ -5455,105 +5463,105 @@
         <v>34.008132371032296</v>
       </c>
     </row>
-    <row r="7" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="76"/>
+    <row r="7" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="81"/>
       <c r="C7" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="85">
+      <c r="D7" s="56">
         <v>550</v>
       </c>
-      <c r="E7" s="85">
+      <c r="E7" s="56">
         <v>357.28</v>
       </c>
-      <c r="F7" s="85">
+      <c r="F7" s="56">
         <v>25.315999999999999</v>
       </c>
-      <c r="G7" s="85">
+      <c r="G7" s="56">
         <v>12.817</v>
       </c>
-      <c r="H7" s="85">
+      <c r="H7" s="56">
         <v>4.0009999999999994</v>
       </c>
-      <c r="I7" s="85">
+      <c r="I7" s="56">
         <v>21.545000000000002</v>
       </c>
-      <c r="J7" s="85">
+      <c r="J7" s="56">
         <v>12.845000000000001</v>
       </c>
-      <c r="K7" s="85">
+      <c r="K7" s="56">
         <v>16.672000000000001</v>
       </c>
-      <c r="L7" s="85">
+      <c r="L7" s="56">
         <v>17.965999999999998</v>
       </c>
-      <c r="M7" s="85">
+      <c r="M7" s="56">
         <v>46.100999999999999</v>
       </c>
-      <c r="N7" s="85">
+      <c r="N7" s="56">
         <v>23.463999999999999</v>
       </c>
-      <c r="O7" s="85">
+      <c r="O7" s="56">
         <v>14.95</v>
       </c>
-      <c r="P7" s="85">
+      <c r="P7" s="56">
         <v>0.89999999999999991</v>
       </c>
-      <c r="Q7" s="85">
+      <c r="Q7" s="56">
         <v>0.89999999999999991</v>
       </c>
-      <c r="R7" s="85">
+      <c r="R7" s="56">
         <v>1.2</v>
       </c>
-      <c r="S7" s="85">
+      <c r="S7" s="56">
         <v>0.70000000000000007</v>
       </c>
-      <c r="T7" s="86">
+      <c r="T7" s="57">
         <v>3.2</v>
       </c>
-      <c r="U7" s="86">
+      <c r="U7" s="57">
         <v>35.699999999999996</v>
       </c>
-      <c r="V7" s="86">
+      <c r="V7" s="57">
         <v>29.299999999999997</v>
       </c>
-      <c r="W7" s="86">
+      <c r="W7" s="57">
         <v>4.7</v>
       </c>
-      <c r="X7" s="86">
+      <c r="X7" s="57">
         <v>11.4</v>
       </c>
-      <c r="Y7" s="86">
+      <c r="Y7" s="57">
         <v>9</v>
       </c>
-      <c r="Z7" s="86">
+      <c r="Z7" s="57">
         <v>9.3000000000000007</v>
       </c>
-      <c r="AA7" s="86">
+      <c r="AA7" s="57">
         <v>19.900000000000002</v>
       </c>
-      <c r="AB7" s="86">
+      <c r="AB7" s="57">
         <v>17.7</v>
       </c>
-      <c r="AC7" s="86">
+      <c r="AC7" s="57">
         <v>7.3999999999999995</v>
       </c>
     </row>
-    <row r="8" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B8" s="76"/>
+    <row r="8" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="81"/>
       <c r="C8" s="38" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="87">
+      <c r="D8" s="58">
         <v>9.9800251535097892</v>
       </c>
-      <c r="E8" s="87">
+      <c r="E8" s="58">
         <v>5.7385981434146682</v>
       </c>
-      <c r="F8" s="87">
+      <c r="F8" s="58">
         <v>1.9613082173916221</v>
       </c>
-      <c r="G8" s="87">
+      <c r="G8" s="58">
         <v>9.8156906297965385</v>
       </c>
       <c r="H8" s="42">
@@ -5623,24 +5631,24 @@
         <v>6.41</v>
       </c>
     </row>
-    <row r="9" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B9" s="76"/>
+    <row r="9" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="81"/>
       <c r="C9" s="38" t="s">
         <v>5</v>
       </c>
-      <c r="D9" s="87">
+      <c r="D9" s="58">
         <v>3.8995298028471241</v>
       </c>
-      <c r="E9" s="87">
+      <c r="E9" s="58">
         <v>3.342855067494094</v>
       </c>
-      <c r="F9" s="87">
+      <c r="F9" s="58">
         <v>1.9925854245399319</v>
       </c>
-      <c r="G9" s="87">
+      <c r="G9" s="58">
         <v>7.4497001400736584</v>
       </c>
-      <c r="H9" s="87">
+      <c r="H9" s="58">
         <v>12.25071028943913</v>
       </c>
       <c r="I9" s="42">
@@ -5707,8 +5715,8 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="10" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="76"/>
+    <row r="10" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="81"/>
       <c r="C10" s="38" t="s">
         <v>36</v>
       </c>
@@ -5725,51 +5733,51 @@
       <c r="N10" s="42"/>
       <c r="O10" s="42"/>
       <c r="P10" s="42"/>
-      <c r="Q10" s="85">
+      <c r="Q10" s="56">
         <v>2.8000000000000003</v>
       </c>
-      <c r="R10" s="85">
+      <c r="R10" s="56">
         <v>1.3</v>
       </c>
-      <c r="S10" s="85">
+      <c r="S10" s="56">
         <v>0.3</v>
       </c>
-      <c r="T10" s="86">
+      <c r="T10" s="57">
         <v>1.2</v>
       </c>
-      <c r="U10" s="86">
+      <c r="U10" s="57">
         <v>6.1</v>
       </c>
-      <c r="V10" s="86">
+      <c r="V10" s="57">
         <v>3.2</v>
       </c>
-      <c r="W10" s="86">
+      <c r="W10" s="57">
         <v>3.1</v>
       </c>
-      <c r="X10" s="86">
+      <c r="X10" s="57">
         <v>4.8</v>
       </c>
-      <c r="Y10" s="86">
+      <c r="Y10" s="57">
         <v>5.7</v>
       </c>
-      <c r="Z10" s="86">
+      <c r="Z10" s="57">
         <v>6.1</v>
       </c>
-      <c r="AA10" s="86">
+      <c r="AA10" s="57">
         <v>6.6000000000000005</v>
       </c>
-      <c r="AB10" s="86">
+      <c r="AB10" s="57">
         <v>5.6000000000000005</v>
       </c>
-      <c r="AC10" s="86">
+      <c r="AC10" s="57">
         <v>5.0999999999999996</v>
       </c>
       <c r="AE10" s="34">
         <v>100</v>
       </c>
     </row>
-    <row r="11" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="76"/>
+    <row r="11" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="81"/>
       <c r="C11" s="38" t="s">
         <v>6</v>
       </c>
@@ -5782,13 +5790,13 @@
       <c r="J11" s="42"/>
       <c r="K11" s="42"/>
       <c r="L11" s="42"/>
-      <c r="M11" s="87">
+      <c r="M11" s="58">
         <v>5.0062736153404677</v>
       </c>
-      <c r="N11" s="87">
+      <c r="N11" s="58">
         <v>1.1696218030110821</v>
       </c>
-      <c r="O11" s="87">
+      <c r="O11" s="58">
         <v>46.8521757193597</v>
       </c>
       <c r="P11" s="42">
@@ -5830,8 +5838,8 @@
       <c r="AB11" s="43"/>
       <c r="AC11" s="43"/>
     </row>
-    <row r="12" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B12" s="76"/>
+    <row r="12" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="81"/>
       <c r="C12" s="38" t="s">
         <v>7</v>
       </c>
@@ -5914,92 +5922,92 @@
         <v>4.0408222020069662</v>
       </c>
     </row>
-    <row r="13" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="76"/>
+    <row r="13" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="81"/>
       <c r="C13" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="D13" s="85">
+      <c r="D13" s="56">
         <v>3.3920215851299802</v>
       </c>
-      <c r="E13" s="85">
+      <c r="E13" s="56">
         <v>1.865125240847725</v>
       </c>
-      <c r="F13" s="85">
+      <c r="F13" s="56">
         <v>-0.28750851176519637</v>
       </c>
-      <c r="G13" s="85">
+      <c r="G13" s="56">
         <v>8.6804765156688362</v>
       </c>
-      <c r="H13" s="85">
+      <c r="H13" s="56">
         <v>3.7212874397822842</v>
       </c>
-      <c r="I13" s="85">
+      <c r="I13" s="56">
         <v>8.4487264229953212</v>
       </c>
-      <c r="J13" s="85">
+      <c r="J13" s="56">
         <v>7.3106761356186372</v>
       </c>
-      <c r="K13" s="85">
+      <c r="K13" s="56">
         <v>6.138510832850498</v>
       </c>
-      <c r="L13" s="85">
+      <c r="L13" s="56">
         <v>12.050855548288551</v>
       </c>
-      <c r="M13" s="85">
+      <c r="M13" s="56">
         <v>13.017256188918539</v>
       </c>
-      <c r="N13" s="85">
+      <c r="N13" s="56">
         <v>3.976552884781682</v>
       </c>
-      <c r="O13" s="85">
+      <c r="O13" s="56">
         <v>16.564349617451519</v>
       </c>
-      <c r="P13" s="85">
+      <c r="P13" s="56">
         <v>12.679037722465891</v>
       </c>
-      <c r="Q13" s="85">
+      <c r="Q13" s="56">
         <v>4.9052087569455676</v>
       </c>
-      <c r="R13" s="85">
+      <c r="R13" s="56">
         <v>3.075706689586414</v>
       </c>
-      <c r="S13" s="85">
+      <c r="S13" s="56">
         <v>5.589686062517254</v>
       </c>
-      <c r="T13" s="86">
+      <c r="T13" s="57">
         <v>5.7063750461621199</v>
       </c>
-      <c r="U13" s="86">
+      <c r="U13" s="57">
         <v>5.2097170591420916</v>
       </c>
-      <c r="V13" s="86">
+      <c r="V13" s="57">
         <v>2.6160119095227441</v>
       </c>
-      <c r="W13" s="86">
+      <c r="W13" s="57">
         <v>2.8675880344689988</v>
       </c>
-      <c r="X13" s="86">
+      <c r="X13" s="57">
         <v>3.313322895445018</v>
       </c>
-      <c r="Y13" s="86">
+      <c r="Y13" s="57">
         <v>2.204572047574139</v>
       </c>
-      <c r="Z13" s="86">
+      <c r="Z13" s="57">
         <v>7.1957888597581032</v>
       </c>
-      <c r="AA13" s="86">
+      <c r="AA13" s="57">
         <v>5.3509480428039531</v>
       </c>
-      <c r="AB13" s="86">
+      <c r="AB13" s="57">
         <v>3.323380336918186</v>
       </c>
-      <c r="AC13" s="86">
+      <c r="AC13" s="57">
         <v>3.5808278443806651</v>
       </c>
     </row>
-    <row r="14" spans="2:31" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B14" s="77"/>
+    <row r="14" spans="2:31" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="82"/>
       <c r="C14" s="39"/>
       <c r="D14" s="44"/>
       <c r="E14" s="44"/>
@@ -6028,47 +6036,47 @@
       <c r="AB14" s="44"/>
       <c r="AC14" s="44"/>
     </row>
-    <row r="15" spans="2:31" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B15" s="81" t="s">
+    <row r="15" spans="2:31" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="86" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="84" t="s">
+      <c r="C15" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="85">
+      <c r="D15" s="56">
         <v>2.7389719231943985</v>
       </c>
-      <c r="E15" s="85">
+      <c r="E15" s="56">
         <v>1.3302515753756454</v>
       </c>
-      <c r="F15" s="85">
+      <c r="F15" s="56">
         <v>4.4337848919472993</v>
       </c>
-      <c r="G15" s="85">
+      <c r="G15" s="56">
         <v>4.1706106631213133</v>
       </c>
-      <c r="H15" s="85">
+      <c r="H15" s="56">
         <v>3.144422693260819</v>
       </c>
-      <c r="I15" s="85">
+      <c r="I15" s="56">
         <v>3.5091522652556395</v>
       </c>
-      <c r="J15" s="85">
+      <c r="J15" s="56">
         <v>3.41826519192416</v>
       </c>
-      <c r="K15" s="85">
+      <c r="K15" s="56">
         <v>4.7150166604238972</v>
       </c>
-      <c r="L15" s="85">
+      <c r="L15" s="56">
         <v>5.2482812574075135</v>
       </c>
-      <c r="M15" s="85">
+      <c r="M15" s="56">
         <v>7.2062322125277003</v>
       </c>
-      <c r="N15" s="85">
+      <c r="N15" s="56">
         <v>6.4405537763731884</v>
       </c>
-      <c r="O15" s="85">
+      <c r="O15" s="56">
         <v>4.4862599971829136</v>
       </c>
       <c r="P15" s="42">
@@ -6114,9 +6122,9 @@
         <v>2.0438541684263956</v>
       </c>
     </row>
-    <row r="16" spans="2:31" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B16" s="82"/>
-      <c r="C16" s="84" t="s">
+    <row r="16" spans="2:31" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="87"/>
+      <c r="C16" s="55" t="s">
         <v>35</v>
       </c>
       <c r="D16" s="45"/>
@@ -6124,111 +6132,111 @@
       <c r="F16" s="45"/>
       <c r="G16" s="45"/>
       <c r="H16" s="45"/>
-      <c r="I16" s="87">
+      <c r="I16" s="58">
         <v>0.40453328581708042</v>
       </c>
-      <c r="J16" s="87">
+      <c r="J16" s="58">
         <v>0.48422407635711356</v>
       </c>
-      <c r="K16" s="87">
+      <c r="K16" s="58">
         <v>0.31416699180356494</v>
       </c>
-      <c r="L16" s="87">
+      <c r="L16" s="58">
         <v>0.10524895577847315</v>
       </c>
-      <c r="M16" s="87">
+      <c r="M16" s="58">
         <v>1.6410530378671728</v>
       </c>
-      <c r="N16" s="87">
+      <c r="N16" s="58">
         <v>1.3071682584986068</v>
       </c>
-      <c r="O16" s="87">
+      <c r="O16" s="58">
         <v>1.1636413073589249</v>
       </c>
-      <c r="P16" s="87">
+      <c r="P16" s="58">
         <v>1.6224631901067894</v>
       </c>
-      <c r="Q16" s="87">
+      <c r="Q16" s="58">
         <v>1.2260230788808939</v>
       </c>
-      <c r="R16" s="87">
+      <c r="R16" s="58">
         <v>1.1322860598496596</v>
       </c>
-      <c r="S16" s="87">
+      <c r="S16" s="58">
         <v>1.0430266435877029</v>
       </c>
-      <c r="T16" s="88">
+      <c r="T16" s="59">
         <v>0.57154452690598689</v>
       </c>
-      <c r="U16" s="88">
+      <c r="U16" s="59">
         <v>0.58950064275132985</v>
       </c>
-      <c r="V16" s="88">
+      <c r="V16" s="59">
         <v>0.40822928255594521</v>
       </c>
-      <c r="W16" s="88">
+      <c r="W16" s="59">
         <v>0.77878679461987477</v>
       </c>
-      <c r="X16" s="88">
+      <c r="X16" s="59">
         <v>0.56013368762434412</v>
       </c>
-      <c r="Y16" s="88">
+      <c r="Y16" s="59">
         <v>1.7098043778173746</v>
       </c>
-      <c r="Z16" s="88">
+      <c r="Z16" s="59">
         <v>1.5317903896834451</v>
       </c>
-      <c r="AA16" s="88">
+      <c r="AA16" s="59">
         <v>1.6903944508226811</v>
       </c>
       <c r="AB16" s="46"/>
       <c r="AC16" s="46"/>
     </row>
-    <row r="17" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B17" s="82"/>
-      <c r="C17" s="84" t="s">
+    <row r="17" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="87"/>
+      <c r="C17" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="87">
+      <c r="D17" s="58">
         <v>2.7341115498508834</v>
       </c>
-      <c r="E17" s="87">
+      <c r="E17" s="58">
         <v>3.0311542200386903</v>
       </c>
-      <c r="F17" s="87">
+      <c r="F17" s="58">
         <v>3.1680904554305527</v>
       </c>
-      <c r="G17" s="87">
+      <c r="G17" s="58">
         <v>4.0353491552928142</v>
       </c>
-      <c r="H17" s="87">
+      <c r="H17" s="58">
         <v>3.3388280480279078</v>
       </c>
-      <c r="I17" s="87">
+      <c r="I17" s="58">
         <v>3.1195715419037282</v>
       </c>
-      <c r="J17" s="87">
+      <c r="J17" s="58">
         <v>3.4761420127020592</v>
       </c>
-      <c r="K17" s="87">
+      <c r="K17" s="58">
         <v>3.8851427867183381</v>
       </c>
-      <c r="L17" s="87">
+      <c r="L17" s="58">
         <v>2.7031114252703956</v>
       </c>
-      <c r="M17" s="87">
+      <c r="M17" s="58">
         <v>4.0119842682636726</v>
       </c>
-      <c r="N17" s="87">
+      <c r="N17" s="58">
         <v>3.7509659749682318</v>
       </c>
-      <c r="O17" s="87">
+      <c r="O17" s="58">
         <v>3.0588761809607661</v>
       </c>
-      <c r="P17" s="87">
+      <c r="P17" s="58">
         <v>3.6894726118970333</v>
       </c>
-      <c r="Q17" s="87">
+      <c r="Q17" s="58">
         <v>4.1179373956539793</v>
       </c>
       <c r="R17" s="42">
@@ -6268,9 +6276,9 @@
         <v>5.7681311123322816</v>
       </c>
     </row>
-    <row r="18" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="82"/>
-      <c r="C18" s="84" t="s">
+    <row r="18" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="87"/>
+      <c r="C18" s="55" t="s">
         <v>5</v>
       </c>
       <c r="D18" s="42"/>
@@ -6332,9 +6340,9 @@
         <v>4.1223540867584374</v>
       </c>
     </row>
-    <row r="19" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="82"/>
-      <c r="C19" s="84" t="s">
+    <row r="19" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="87"/>
+      <c r="C19" s="55" t="s">
         <v>36</v>
       </c>
       <c r="D19" s="42"/>
@@ -6364,9 +6372,9 @@
       <c r="AB19" s="43"/>
       <c r="AC19" s="43"/>
     </row>
-    <row r="20" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="82"/>
-      <c r="C20" s="84" t="s">
+    <row r="20" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="87"/>
+      <c r="C20" s="55" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="42"/>
@@ -6426,15 +6434,15 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="21" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B21" s="82"/>
-      <c r="C21" s="84" t="s">
+    <row r="21" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B21" s="87"/>
+      <c r="C21" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="D21" s="96">
+      <c r="D21" s="64">
         <v>5.3523295151744685</v>
       </c>
-      <c r="E21" s="96">
+      <c r="E21" s="64">
         <v>5.4638519453679804</v>
       </c>
       <c r="F21" s="42">
@@ -6510,75 +6518,75 @@
         <v>4.3655198743777506</v>
       </c>
     </row>
-    <row r="22" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B22" s="82"/>
-      <c r="C22" s="84" t="s">
+    <row r="22" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="87"/>
+      <c r="C22" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="D22" s="87">
+      <c r="D22" s="58">
         <v>6.160424819339247</v>
       </c>
-      <c r="E22" s="87">
+      <c r="E22" s="58">
         <v>7.1551556497267557</v>
       </c>
-      <c r="F22" s="87">
+      <c r="F22" s="58">
         <v>6.6556843363485401</v>
       </c>
-      <c r="G22" s="87">
+      <c r="G22" s="58">
         <v>7.4645014273508545</v>
       </c>
-      <c r="H22" s="87">
+      <c r="H22" s="58">
         <v>7.0224114634656107</v>
       </c>
-      <c r="I22" s="87">
+      <c r="I22" s="58">
         <v>6.1118215068306307</v>
       </c>
-      <c r="J22" s="87">
+      <c r="J22" s="58">
         <v>6.6105167200113533</v>
       </c>
-      <c r="K22" s="87">
+      <c r="K22" s="58">
         <v>7.2036431622180279</v>
       </c>
-      <c r="L22" s="87">
+      <c r="L22" s="58">
         <v>4.8597339684994392</v>
       </c>
-      <c r="M22" s="87">
+      <c r="M22" s="58">
         <v>6.372568189312859</v>
       </c>
-      <c r="N22" s="87">
+      <c r="N22" s="58">
         <v>4.9957308902738946</v>
       </c>
-      <c r="O22" s="87">
+      <c r="O22" s="58">
         <v>3.9868997528571022</v>
       </c>
-      <c r="P22" s="87">
+      <c r="P22" s="58">
         <v>4.5911146331197648</v>
       </c>
-      <c r="Q22" s="87">
+      <c r="Q22" s="58">
         <v>4.9943084939053648</v>
       </c>
-      <c r="R22" s="87">
+      <c r="R22" s="58">
         <v>4.7567577949389594</v>
       </c>
-      <c r="S22" s="87">
+      <c r="S22" s="58">
         <v>4.4751865664336918</v>
       </c>
-      <c r="T22" s="87">
+      <c r="T22" s="58">
         <v>5.1786766022405004</v>
       </c>
-      <c r="U22" s="87">
+      <c r="U22" s="58">
         <v>5.4923814809478868</v>
       </c>
-      <c r="V22" s="87">
+      <c r="V22" s="58">
         <v>3.987417295453886</v>
       </c>
-      <c r="W22" s="87">
+      <c r="W22" s="58">
         <v>3.6385474330877057</v>
       </c>
-      <c r="X22" s="87">
+      <c r="X22" s="58">
         <v>4.2669440012611952</v>
       </c>
-      <c r="Y22" s="87">
+      <c r="Y22" s="58">
         <v>5.0253060121891853</v>
       </c>
       <c r="Z22" s="42">
@@ -6594,8 +6602,8 @@
         <v>3.6771878487771641</v>
       </c>
     </row>
-    <row r="23" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B23" s="83"/>
+    <row r="23" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="88"/>
       <c r="C23" s="40"/>
       <c r="D23" s="47"/>
       <c r="E23" s="47"/>
@@ -6624,8 +6632,8 @@
       <c r="AB23" s="47"/>
       <c r="AC23" s="47"/>
     </row>
-    <row r="24" spans="2:29" ht="14.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B24" s="78" t="s">
+    <row r="24" spans="2:29" ht="14.55" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="83" t="s">
         <v>59</v>
       </c>
       <c r="C24" s="38" t="s">
@@ -6688,84 +6696,84 @@
         <v>-1.7</v>
       </c>
     </row>
-    <row r="25" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B25" s="79"/>
+    <row r="25" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="84"/>
       <c r="C25" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="D25" s="99">
+      <c r="D25" s="67">
         <v>-0.93646885507273803</v>
       </c>
-      <c r="E25" s="99">
+      <c r="E25" s="67">
         <v>-1.3763341043419501E-2</v>
       </c>
-      <c r="F25" s="99">
+      <c r="F25" s="67">
         <v>0.53120756119524348</v>
       </c>
-      <c r="G25" s="99">
+      <c r="G25" s="67">
         <v>-0.33670775179637491</v>
       </c>
-      <c r="H25" s="99">
+      <c r="H25" s="67">
         <v>-0.63843389275770546</v>
       </c>
-      <c r="I25" s="99">
+      <c r="I25" s="67">
         <v>-0.57297280860683997</v>
       </c>
-      <c r="J25" s="99">
+      <c r="J25" s="67">
         <v>-0.80358628874287008</v>
       </c>
-      <c r="K25" s="99">
+      <c r="K25" s="67">
         <v>-0.58205586807288046</v>
       </c>
-      <c r="L25" s="99">
+      <c r="L25" s="67">
         <v>-5.4705675649268239E-2</v>
       </c>
-      <c r="M25" s="99">
+      <c r="M25" s="67">
         <v>0.25974913985859915</v>
       </c>
-      <c r="N25" s="99">
+      <c r="N25" s="67">
         <v>2.0732940733949414</v>
       </c>
-      <c r="O25" s="99"/>
-      <c r="P25" s="99">
+      <c r="O25" s="67"/>
+      <c r="P25" s="67">
         <v>0.60285156314407162</v>
       </c>
-      <c r="Q25" s="99">
+      <c r="Q25" s="67">
         <v>-0.89908451716650384</v>
       </c>
-      <c r="R25" s="99">
+      <c r="R25" s="67">
         <v>9.322215159772726E-2</v>
       </c>
-      <c r="S25" s="99">
+      <c r="S25" s="67">
         <v>-0.6409321033803228</v>
       </c>
-      <c r="T25" s="100">
+      <c r="T25" s="68">
         <v>-1.2376838778088541</v>
       </c>
-      <c r="U25" s="100">
+      <c r="U25" s="68">
         <v>0.11720742272574117</v>
       </c>
-      <c r="V25" s="100">
+      <c r="V25" s="68">
         <v>-0.73038240096275608</v>
       </c>
-      <c r="W25" s="100">
+      <c r="W25" s="68">
         <v>-0.81307702771113177</v>
       </c>
-      <c r="X25" s="100">
+      <c r="X25" s="68">
         <v>-1.2021592684284059</v>
       </c>
-      <c r="Y25" s="100">
+      <c r="Y25" s="68">
         <v>-0.23194385087152775</v>
       </c>
-      <c r="Z25" s="100">
+      <c r="Z25" s="68">
         <v>-2.069057967448888</v>
       </c>
-      <c r="AA25" s="100"/>
-      <c r="AB25" s="100"/>
-      <c r="AC25" s="100"/>
-    </row>
-    <row r="26" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B26" s="79"/>
+      <c r="AA25" s="68"/>
+      <c r="AB25" s="68"/>
+      <c r="AC25" s="68"/>
+    </row>
+    <row r="26" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="84"/>
       <c r="C26" s="38" t="s">
         <v>10</v>
       </c>
@@ -6848,8 +6856,8 @@
         <v>-7.2560365679833261</v>
       </c>
     </row>
-    <row r="27" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B27" s="79"/>
+    <row r="27" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="84"/>
       <c r="C27" s="38" t="s">
         <v>5</v>
       </c>
@@ -6920,8 +6928,8 @@
         <v>-5.7</v>
       </c>
     </row>
-    <row r="28" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B28" s="79"/>
+    <row r="28" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="84"/>
       <c r="C28" s="38" t="s">
         <v>36</v>
       </c>
@@ -6952,8 +6960,8 @@
       <c r="AB28" s="51"/>
       <c r="AC28" s="51"/>
     </row>
-    <row r="29" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B29" s="79"/>
+    <row r="29" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="84"/>
       <c r="C29" s="38" t="s">
         <v>6</v>
       </c>
@@ -7012,8 +7020,8 @@
         <v>2.5569999999999999</v>
       </c>
     </row>
-    <row r="30" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="79"/>
+    <row r="30" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="84"/>
       <c r="C30" s="38" t="s">
         <v>7</v>
       </c>
@@ -7096,8 +7104,8 @@
         <v>-2.5324702348127164</v>
       </c>
     </row>
-    <row r="31" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B31" s="79"/>
+    <row r="31" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="84"/>
       <c r="C31" s="38" t="s">
         <v>8</v>
       </c>
@@ -7116,40 +7124,40 @@
       <c r="P31" s="42"/>
       <c r="Q31" s="42"/>
       <c r="R31" s="42"/>
-      <c r="S31" s="87">
+      <c r="S31" s="58">
         <v>-2.1126936142681005</v>
       </c>
-      <c r="T31" s="87">
+      <c r="T31" s="58">
         <v>-2.2369945879372302</v>
       </c>
-      <c r="U31" s="87">
+      <c r="U31" s="58">
         <v>-2.4546632646083708</v>
       </c>
-      <c r="V31" s="87">
+      <c r="V31" s="58">
         <v>-2.6656185792822731</v>
       </c>
-      <c r="W31" s="98">
+      <c r="W31" s="66">
         <v>-3.4475281309551931</v>
       </c>
-      <c r="X31" s="87">
+      <c r="X31" s="58">
         <v>-6.139323520204595</v>
       </c>
-      <c r="Y31" s="87">
+      <c r="Y31" s="58">
         <v>-7.9313040173589355</v>
       </c>
-      <c r="Z31" s="87">
+      <c r="Z31" s="58">
         <v>-6.7428490151198419</v>
       </c>
-      <c r="AA31" s="87">
+      <c r="AA31" s="58">
         <v>-4.9423963934475452</v>
       </c>
-      <c r="AB31" s="87">
+      <c r="AB31" s="58">
         <v>-4.3234415146220666</v>
       </c>
       <c r="AC31" s="42"/>
     </row>
-    <row r="32" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B32" s="80"/>
+    <row r="32" spans="2:29" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="85"/>
       <c r="C32" s="38"/>
       <c r="D32" s="44"/>
       <c r="E32" s="44"/>
@@ -7178,11 +7186,11 @@
       <c r="AB32" s="44"/>
       <c r="AC32" s="44"/>
     </row>
-    <row r="33" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B33" s="73" t="s">
+    <row r="33" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="89" t="s">
         <v>61</v>
       </c>
-      <c r="C33" s="84" t="s">
+      <c r="C33" s="55" t="s">
         <v>4</v>
       </c>
       <c r="D33" s="42"/>
@@ -7244,9 +7252,9 @@
         <v>42.505624189722383</v>
       </c>
     </row>
-    <row r="34" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B34" s="74"/>
-      <c r="C34" s="84" t="s">
+    <row r="34" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="90"/>
+      <c r="C34" s="55" t="s">
         <v>35</v>
       </c>
       <c r="D34" s="45"/>
@@ -7276,9 +7284,9 @@
       <c r="AB34" s="46"/>
       <c r="AC34" s="46"/>
     </row>
-    <row r="35" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="74"/>
-      <c r="C35" s="84" t="s">
+    <row r="35" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="90"/>
+      <c r="C35" s="55" t="s">
         <v>10</v>
       </c>
       <c r="D35" s="42">
@@ -7360,9 +7368,9 @@
         <v>65.599999999999994</v>
       </c>
     </row>
-    <row r="36" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="74"/>
-      <c r="C36" s="84" t="s">
+    <row r="36" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="90"/>
+      <c r="C36" s="55" t="s">
         <v>5</v>
       </c>
       <c r="D36" s="42"/>
@@ -7416,9 +7424,9 @@
         <v>53.7</v>
       </c>
     </row>
-    <row r="37" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B37" s="74"/>
-      <c r="C37" s="84" t="s">
+    <row r="37" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="90"/>
+      <c r="C37" s="55" t="s">
         <v>36</v>
       </c>
       <c r="D37" s="42"/>
@@ -7448,9 +7456,9 @@
       <c r="AB37" s="43"/>
       <c r="AC37" s="43"/>
     </row>
-    <row r="38" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B38" s="74"/>
-      <c r="C38" s="84" t="s">
+    <row r="38" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="90"/>
+      <c r="C38" s="55" t="s">
         <v>6</v>
       </c>
       <c r="D38" s="42"/>
@@ -7508,9 +7516,9 @@
         <v>35.183846266442188</v>
       </c>
     </row>
-    <row r="39" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B39" s="74"/>
-      <c r="C39" s="84" t="s">
+    <row r="39" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="90"/>
+      <c r="C39" s="55" t="s">
         <v>7</v>
       </c>
       <c r="D39" s="42"/>
@@ -7518,47 +7526,71 @@
       <c r="F39" s="42"/>
       <c r="G39" s="42"/>
       <c r="H39" s="42"/>
-      <c r="I39" s="42"/>
-      <c r="J39" s="42"/>
-      <c r="K39" s="42"/>
-      <c r="L39" s="42"/>
-      <c r="M39" s="42"/>
-      <c r="N39" s="42"/>
-      <c r="O39" s="42"/>
-      <c r="P39" s="42"/>
-      <c r="Q39" s="42"/>
-      <c r="R39" s="42"/>
-      <c r="S39" s="42"/>
-      <c r="T39" s="43"/>
-      <c r="U39" s="43"/>
+      <c r="I39" s="99"/>
+      <c r="J39" s="42">
+        <v>26.01355257698248</v>
+      </c>
+      <c r="K39" s="42">
+        <v>24.843045603038604</v>
+      </c>
+      <c r="L39" s="42">
+        <v>27.347185316865847</v>
+      </c>
+      <c r="M39" s="42">
+        <v>26.71847721717101</v>
+      </c>
+      <c r="N39" s="42">
+        <v>30.036728996039912</v>
+      </c>
+      <c r="O39" s="42">
+        <v>31.405226763545809</v>
+      </c>
+      <c r="P39" s="42">
+        <v>31.12641104754173</v>
+      </c>
+      <c r="Q39" s="42">
+        <v>32.792783566238072</v>
+      </c>
+      <c r="R39" s="42">
+        <v>31.979521143883339</v>
+      </c>
+      <c r="S39" s="42">
+        <v>36.220840621376361</v>
+      </c>
+      <c r="T39" s="43">
+        <v>39.638294955769467</v>
+      </c>
+      <c r="U39" s="43">
+        <v>39.862863681762803</v>
+      </c>
       <c r="V39" s="43">
-        <v>38</v>
+        <v>38.34438254425482</v>
       </c>
       <c r="W39" s="43">
-        <v>37.799999999999997</v>
+        <v>38.135062390300725</v>
       </c>
       <c r="X39" s="43">
-        <v>39.9</v>
+        <v>40.225518904658173</v>
       </c>
       <c r="Y39" s="43">
-        <v>40.299999999999997</v>
+        <v>40.597540762039621</v>
       </c>
       <c r="Z39" s="43">
-        <v>42.4</v>
+        <v>42.748780817726285</v>
       </c>
       <c r="AA39" s="43">
-        <v>45.4</v>
+        <v>45.520785186582543</v>
       </c>
       <c r="AB39" s="43">
-        <v>49</v>
+        <v>49.046233536837555</v>
       </c>
       <c r="AC39" s="43">
-        <v>46.2</v>
-      </c>
-    </row>
-    <row r="40" spans="2:29" ht="14.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B40" s="74"/>
-      <c r="C40" s="84" t="s">
+        <v>46.496916095886149</v>
+      </c>
+    </row>
+    <row r="40" spans="2:29" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="90"/>
+      <c r="C40" s="55" t="s">
         <v>8</v>
       </c>
       <c r="D40" s="42"/>
@@ -7579,31 +7611,31 @@
       <c r="S40" s="42"/>
       <c r="T40" s="42"/>
       <c r="U40" s="42"/>
-      <c r="V40" s="88">
+      <c r="V40" s="59">
         <v>34.67357099456936</v>
       </c>
-      <c r="W40" s="88">
+      <c r="W40" s="59">
         <v>38.476945312033109</v>
       </c>
-      <c r="X40" s="87">
+      <c r="X40" s="58">
         <v>44.185914308992402</v>
       </c>
-      <c r="Y40" s="87">
+      <c r="Y40" s="58">
         <v>51.30266235001956</v>
       </c>
-      <c r="Z40" s="87">
+      <c r="Z40" s="58">
         <v>53.890283064003967</v>
       </c>
-      <c r="AA40" s="87">
+      <c r="AA40" s="58">
         <v>53.146935074866661</v>
       </c>
-      <c r="AB40" s="87">
+      <c r="AB40" s="58">
         <v>54.430552583667115</v>
       </c>
       <c r="AC40" s="42"/>
     </row>
-    <row r="41" spans="2:29" x14ac:dyDescent="0.3">
-      <c r="B41" s="75"/>
+    <row r="41" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="B41" s="91"/>
       <c r="C41" s="41"/>
       <c r="D41" s="53"/>
       <c r="E41" s="53"/>
@@ -7632,7 +7664,7 @@
       <c r="AB41" s="53"/>
       <c r="AC41" s="53"/>
     </row>
-    <row r="42" spans="2:29" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:29" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B42" s="36"/>
       <c r="C42" s="37"/>
       <c r="D42" s="37"/>
@@ -7661,7 +7693,7 @@
       <c r="AB42" s="37"/>
       <c r="AC42" s="37"/>
     </row>
-    <row r="43" spans="2:29" ht="16" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:29" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B43" s="36"/>
       <c r="C43" s="37"/>
       <c r="D43" s="37"/>
@@ -7690,14 +7722,31 @@
       <c r="AB43" s="37"/>
       <c r="AC43" s="37"/>
     </row>
-    <row r="44" spans="2:29" ht="16" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:29" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B44" s="36"/>
     </row>
-    <row r="45" spans="2:29" ht="16" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:29" ht="16.8" x14ac:dyDescent="0.25">
       <c r="B45" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="B1:Y1"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="I4:I5"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="V4:V5"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="N4:N5"/>
+    <mergeCell ref="O4:O5"/>
+    <mergeCell ref="P4:P5"/>
     <mergeCell ref="AC4:AC5"/>
     <mergeCell ref="B6:B14"/>
     <mergeCell ref="B15:B23"/>
@@ -7714,23 +7763,6 @@
     <mergeCell ref="S4:S5"/>
     <mergeCell ref="T4:T5"/>
     <mergeCell ref="U4:U5"/>
-    <mergeCell ref="V4:V5"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="L4:L5"/>
-    <mergeCell ref="M4:M5"/>
-    <mergeCell ref="N4:N5"/>
-    <mergeCell ref="O4:O5"/>
-    <mergeCell ref="P4:P5"/>
-    <mergeCell ref="B1:Y1"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="J4:J5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
@@ -7738,210 +7770,209 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26" style="56" customWidth="1"/>
-    <col min="2" max="2" width="30" style="56" customWidth="1"/>
-    <col min="3" max="4" width="40" style="56" customWidth="1"/>
-    <col min="5" max="16384" width="8.7265625" style="56"/>
+    <col min="1" max="1" width="26" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="89" t="s">
+    <row r="1" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="97" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
-      <c r="D1" s="70"/>
-    </row>
-    <row r="2" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="90" t="s">
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+    </row>
+    <row r="2" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="98" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="70"/>
-      <c r="C2" s="70"/>
-      <c r="D2" s="70"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="91" t="s">
+      <c r="B2" s="93"/>
+      <c r="C2" s="93"/>
+      <c r="D2" s="93"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="B4" s="91" t="s">
+      <c r="B4" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="C4" s="91" t="s">
+      <c r="C4" s="60" t="s">
         <v>66</v>
       </c>
-      <c r="D4" s="91" t="s">
+      <c r="D4" s="60" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="90" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="98" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="70"/>
-      <c r="C5" s="70"/>
-      <c r="D5" s="70"/>
-    </row>
-    <row r="6" spans="1:4" ht="25" x14ac:dyDescent="0.35">
-      <c r="A6" s="92" t="s">
+      <c r="B5" s="93"/>
+      <c r="C5" s="93"/>
+      <c r="D5" s="93"/>
+    </row>
+    <row r="6" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A6" s="61" t="s">
         <v>69</v>
       </c>
-      <c r="B6" s="92" t="s">
+      <c r="B6" s="61" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="92" t="s">
+      <c r="C6" s="61" t="s">
         <v>71</v>
       </c>
-      <c r="D6" s="93" t="s">
+      <c r="D6" s="62" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A7" s="92" t="s">
+    <row r="7" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="61" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="92" t="s">
+      <c r="B7" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="92" t="s">
+      <c r="C7" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="97" t="s">
+      <c r="D7" s="65" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="25" x14ac:dyDescent="0.35">
-      <c r="A8" s="92" t="s">
+    <row r="8" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A8" s="61" t="s">
         <v>77</v>
       </c>
-      <c r="B8" s="92" t="s">
+      <c r="B8" s="61" t="s">
         <v>78</v>
       </c>
-      <c r="C8" s="92" t="s">
+      <c r="C8" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="93" t="s">
+      <c r="D8" s="62" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="25" x14ac:dyDescent="0.35">
-      <c r="A9" s="92" t="s">
+    <row r="9" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A9" s="61" t="s">
         <v>80</v>
       </c>
-      <c r="B9" s="92" t="s">
+      <c r="B9" s="61" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="92" t="s">
+      <c r="C9" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="D9" s="93" t="s">
+      <c r="D9" s="62" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="25" x14ac:dyDescent="0.35">
-      <c r="A10" s="92" t="s">
+    <row r="10" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="61" t="s">
         <v>83</v>
       </c>
-      <c r="B10" s="92" t="s">
+      <c r="B10" s="61" t="s">
         <v>84</v>
       </c>
-      <c r="C10" s="92" t="s">
+      <c r="C10" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="D10" s="93" t="s">
+      <c r="D10" s="62" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A11" s="92" t="s">
+    <row r="11" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="61" t="s">
         <v>86</v>
       </c>
-      <c r="B11" s="92" t="s">
+      <c r="B11" s="61" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="92" t="s">
+      <c r="C11" s="61" t="s">
         <v>88</v>
       </c>
-      <c r="D11" s="93" t="s">
+      <c r="D11" s="62" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="37.5" x14ac:dyDescent="0.35">
-      <c r="A12" s="92" t="s">
+    <row r="12" spans="1:4" ht="39.6" x14ac:dyDescent="0.3">
+      <c r="A12" s="61" t="s">
         <v>90</v>
       </c>
-      <c r="B12" s="92" t="s">
+      <c r="B12" s="61" t="s">
         <v>91</v>
       </c>
-      <c r="C12" s="92" t="s">
+      <c r="C12" s="61" t="s">
         <v>92</v>
       </c>
-      <c r="D12" s="93" t="s">
+      <c r="D12" s="62" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="25" x14ac:dyDescent="0.35">
-      <c r="A13" s="92" t="s">
+    <row r="13" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="A13" s="61" t="s">
         <v>94</v>
       </c>
-      <c r="B13" s="92" t="s">
+      <c r="B13" s="61" t="s">
         <v>95</v>
       </c>
-      <c r="C13" s="92" t="s">
+      <c r="C13" s="61" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="93" t="s">
+      <c r="D13" s="62" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="94" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="63" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="95" t="s">
+    <row r="17" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="96" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="70"/>
-      <c r="C17" s="70"/>
-      <c r="D17" s="70"/>
-    </row>
-    <row r="18" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="95" t="s">
+      <c r="B17" s="93"/>
+      <c r="C17" s="93"/>
+      <c r="D17" s="93"/>
+    </row>
+    <row r="18" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="96" t="s">
         <v>100</v>
       </c>
-      <c r="B18" s="70"/>
-      <c r="C18" s="70"/>
-      <c r="D18" s="70"/>
-    </row>
-    <row r="19" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="95" t="s">
+      <c r="B18" s="93"/>
+      <c r="C18" s="93"/>
+      <c r="D18" s="93"/>
+    </row>
+    <row r="19" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="96" t="s">
         <v>101</v>
       </c>
-      <c r="B19" s="70"/>
-      <c r="C19" s="70"/>
-      <c r="D19" s="70"/>
-    </row>
-    <row r="20" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="95" t="s">
+      <c r="B19" s="93"/>
+      <c r="C19" s="93"/>
+      <c r="D19" s="93"/>
+    </row>
+    <row r="20" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="96" t="s">
         <v>102</v>
       </c>
-      <c r="B20" s="70"/>
-      <c r="C20" s="70"/>
-      <c r="D20" s="70"/>
-    </row>
-    <row r="21" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="95" t="s">
+      <c r="B20" s="93"/>
+      <c r="C20" s="93"/>
+      <c r="D20" s="93"/>
+    </row>
+    <row r="21" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="96" t="s">
         <v>103</v>
       </c>
-      <c r="B21" s="70"/>
-      <c r="C21" s="70"/>
-      <c r="D21" s="70"/>
+      <c r="B21" s="93"/>
+      <c r="C21" s="93"/>
+      <c r="D21" s="93"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -7955,12 +7986,12 @@
     <mergeCell ref="A19:D19"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="D6" r:id="rId1"/>
-    <hyperlink ref="D7" r:id="rId2"/>
-    <hyperlink ref="D8" r:id="rId3"/>
-    <hyperlink ref="D9" r:id="rId4"/>
-    <hyperlink ref="D10" r:id="rId5"/>
-    <hyperlink ref="D11" r:id="rId6"/>
+    <hyperlink ref="D6" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="D7" r:id="rId2" xr:uid="{00000000-0004-0000-0300-000001000000}"/>
+    <hyperlink ref="D8" r:id="rId3" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
+    <hyperlink ref="D9" r:id="rId4" xr:uid="{00000000-0004-0000-0300-000003000000}"/>
+    <hyperlink ref="D10" r:id="rId5" xr:uid="{00000000-0004-0000-0300-000004000000}"/>
+    <hyperlink ref="D11" r:id="rId6" xr:uid="{00000000-0004-0000-0300-000005000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>